<commit_message>
[수정] 권한 명칭 변경 (Auth > Role)
</commit_message>
<xml_diff>
--- a/02.프로젝트/01.인트라넷/01.설계/인트라넷 데이터.xlsx
+++ b/02.프로젝트/01.인트라넷/01.설계/인트라넷 데이터.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\knn\Documents\hikr90\02.프로젝트\01.인트라넷\01.설계\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3306B86-95C3-4B2A-96F8-F22920459A16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1B3395A-18C3-4DA2-9392-8732BFA29734}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="793" xr2:uid="{B204C4DA-9ED1-4F0A-AC7E-C11DE778500E}"/>
   </bookViews>
   <sheets>
     <sheet name="MENU" sheetId="8" r:id="rId1"/>
-    <sheet name="AUTH" sheetId="20" r:id="rId2"/>
-    <sheet name="MENU_AUTH" sheetId="21" r:id="rId3"/>
-    <sheet name="EMP_AUTH" sheetId="24" r:id="rId4"/>
+    <sheet name="ROLE" sheetId="20" r:id="rId2"/>
+    <sheet name="MENU_ROLE" sheetId="21" r:id="rId3"/>
+    <sheet name="EMP_ROLE" sheetId="24" r:id="rId4"/>
     <sheet name="EMPINFO" sheetId="22" r:id="rId5"/>
     <sheet name="ORG" sheetId="25" r:id="rId6"/>
     <sheet name="RANK" sheetId="26" r:id="rId7"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="562" uniqueCount="276">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="562" uniqueCount="278">
   <si>
     <t>EMP_IDX</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -147,18 +147,6 @@
     <t>intrBoardInqy1010.do</t>
   </si>
   <si>
-    <t>AUTH_CD</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>AUTH_NM</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>AUTH_0001</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>관리자 권한</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -232,21 +220,12 @@
     <t>권한 관리</t>
   </si>
   <si>
-    <t>intrAuthInqy1010.do</t>
-  </si>
-  <si>
     <t>메뉴 권한 부여</t>
   </si>
   <si>
-    <t>intrAuthInqy2010.do</t>
-  </si>
-  <si>
     <t>사용자 권한 부여</t>
   </si>
   <si>
-    <t>intrAuthInqy3010.do</t>
-  </si>
-  <si>
     <t>MENU_0022</t>
   </si>
   <si>
@@ -263,26 +242,11 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>AUTH</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>intrProjInqy1010.do</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>AUTH_0002</t>
-  </si>
-  <si>
     <t>테스트 권한</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>MENU_AUTH</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>EMP_AUTH</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -1238,6 +1202,45 @@
   <si>
     <t>결재양식 관리</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ROLE</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ROLE_CD</t>
+  </si>
+  <si>
+    <t>ROLE_CD</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ROLE_0001</t>
+  </si>
+  <si>
+    <t>ROLE_0001</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ROLE_NM</t>
+  </si>
+  <si>
+    <t>ROLE_0002</t>
+  </si>
+  <si>
+    <t>EMP_ROLE</t>
+  </si>
+  <si>
+    <t>MENU_ROLE</t>
+  </si>
+  <si>
+    <t>intrRoleInqy1010.do</t>
+  </si>
+  <si>
+    <t>intrRoleInqy2010.do</t>
+  </si>
+  <si>
+    <t>intrRoleInqy3010.do</t>
   </si>
 </sst>
 </file>
@@ -1676,7 +1679,7 @@
   <sheetData>
     <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -1714,18 +1717,18 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B3" s="4">
         <v>0</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="D3" s="4"/>
       <c r="E3" s="4"/>
       <c r="F3" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G3" s="4">
         <v>1</v>
@@ -1744,16 +1747,16 @@
         <v>0</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G4" s="4">
         <v>2</v>
@@ -1772,16 +1775,16 @@
         <v>0</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>189</v>
+        <v>179</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G5" s="4">
         <v>3</v>
@@ -1800,16 +1803,16 @@
         <v>0</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>273</v>
+        <v>263</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>240</v>
+        <v>230</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G6" s="4">
         <v>4</v>
@@ -1828,16 +1831,16 @@
         <v>0</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>272</v>
+        <v>262</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>274</v>
+        <v>264</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G7" s="4">
         <v>5</v>
@@ -1856,12 +1859,12 @@
         <v>0</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D8" s="4"/>
       <c r="E8" s="4"/>
       <c r="F8" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G8" s="4">
         <v>6</v>
@@ -1880,16 +1883,16 @@
         <v>0</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
       <c r="D9" s="4" t="s">
         <v>19</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G9" s="4">
         <v>7</v>
@@ -1908,16 +1911,16 @@
         <v>0</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="D10" s="4" t="s">
         <v>19</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G10" s="4">
         <v>8</v>
@@ -1936,16 +1939,16 @@
         <v>0</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>214</v>
+        <v>204</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>19</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>258</v>
+        <v>248</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G11" s="4">
         <v>9</v>
@@ -1964,12 +1967,12 @@
         <v>0</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>242</v>
+        <v>232</v>
       </c>
       <c r="D12" s="4"/>
       <c r="E12" s="4"/>
       <c r="F12" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G12" s="4">
         <v>10</v>
@@ -1988,16 +1991,16 @@
         <v>0</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>152</v>
+        <v>142</v>
       </c>
       <c r="D13" s="4" t="s">
         <v>23</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G13" s="4">
         <v>11</v>
@@ -2016,16 +2019,16 @@
         <v>0</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
       <c r="D14" s="4" t="s">
         <v>23</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>241</v>
+        <v>231</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G14" s="4">
         <v>12</v>
@@ -2044,12 +2047,12 @@
         <v>0</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D15" s="4"/>
       <c r="E15" s="4"/>
       <c r="F15" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G15" s="4">
         <v>13</v>
@@ -2068,16 +2071,16 @@
         <v>0</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>207</v>
+        <v>197</v>
       </c>
       <c r="D16" s="4" t="s">
         <v>26</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G16" s="4">
         <v>14</v>
@@ -2096,16 +2099,16 @@
         <v>0</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>215</v>
+        <v>205</v>
       </c>
       <c r="D17" s="4" t="s">
         <v>26</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>216</v>
+        <v>206</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G17" s="4">
         <v>15</v>
@@ -2124,12 +2127,12 @@
         <v>1</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="D18" s="4"/>
       <c r="E18" s="4"/>
       <c r="F18" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G18" s="4">
         <v>16</v>
@@ -2148,7 +2151,7 @@
         <v>1</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>29</v>
@@ -2157,7 +2160,7 @@
         <v>31</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G19" s="4">
         <v>17</v>
@@ -2170,22 +2173,22 @@
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B20" s="4">
         <v>1</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>208</v>
+        <v>198</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>29</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>211</v>
+        <v>201</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G20" s="4">
         <v>18</v>
@@ -2198,22 +2201,22 @@
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B21" s="4">
         <v>1</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D21" s="4" t="s">
         <v>29</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G21" s="4">
         <v>19</v>
@@ -2226,18 +2229,18 @@
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B22" s="4">
         <v>1</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>259</v>
+        <v>249</v>
       </c>
       <c r="D22" s="4"/>
       <c r="E22" s="4"/>
       <c r="F22" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G22" s="4">
         <v>20</v>
@@ -2250,22 +2253,22 @@
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B23" s="4">
         <v>1</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>275</v>
+        <v>265</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G23" s="4">
         <v>21</v>
@@ -2278,22 +2281,22 @@
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="B24" s="4">
         <v>1</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G24" s="4">
         <v>23</v>
@@ -2306,18 +2309,18 @@
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="B25" s="4">
         <v>1</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D25" s="4"/>
       <c r="E25" s="4"/>
       <c r="F25" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G25" s="4">
         <v>24</v>
@@ -2330,22 +2333,22 @@
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
-        <v>151</v>
+        <v>141</v>
       </c>
       <c r="B26" s="4">
         <v>1</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G26" s="4">
         <v>25</v>
@@ -2358,22 +2361,22 @@
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="B27" s="4">
         <v>1</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>222</v>
+        <v>212</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>217</v>
+        <v>207</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G27" s="4">
         <v>26</v>
@@ -2386,18 +2389,18 @@
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
-        <v>212</v>
+        <v>202</v>
       </c>
       <c r="B28" s="4">
         <v>1</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="D28" s="4"/>
       <c r="E28" s="4"/>
       <c r="F28" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G28" s="4">
         <v>27</v>
@@ -2410,22 +2413,22 @@
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
-        <v>213</v>
+        <v>203</v>
       </c>
       <c r="B29" s="4">
         <v>1</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>212</v>
+        <v>202</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>59</v>
+        <v>275</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G29" s="4">
         <v>28</v>
@@ -2433,27 +2436,27 @@
       <c r="H29" s="4"/>
       <c r="J29" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>INSERT INTO MENU VALUES('MENU_0027','1','권한 관리','MENU_0026','intrAuthInqy1010.do','Y','28','');</v>
+        <v>INSERT INTO MENU VALUES('MENU_0027','1','권한 관리','MENU_0026','intrRoleInqy1010.do','Y','28','');</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
-        <v>218</v>
+        <v>208</v>
       </c>
       <c r="B30" s="4">
         <v>1</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>212</v>
+        <v>202</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>61</v>
+        <v>276</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G30" s="4">
         <v>29</v>
@@ -2461,27 +2464,27 @@
       <c r="H30" s="4"/>
       <c r="J30" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>INSERT INTO MENU VALUES('MENU_0028','1','메뉴 권한 부여','MENU_0026','intrAuthInqy2010.do','Y','29','');</v>
+        <v>INSERT INTO MENU VALUES('MENU_0028','1','메뉴 권한 부여','MENU_0026','intrRoleInqy2010.do','Y','29','');</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
-        <v>219</v>
+        <v>209</v>
       </c>
       <c r="B31" s="4">
         <v>1</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>212</v>
+        <v>202</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>63</v>
+        <v>277</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G31" s="4">
         <v>30</v>
@@ -2489,27 +2492,27 @@
       <c r="H31" s="4"/>
       <c r="J31" s="3" t="str">
         <f t="shared" ref="J31" si="8">"INSERT INTO "&amp;$A$1&amp;" VALUES('"&amp;A31&amp;"','"&amp;B31&amp;"','"&amp;C31&amp;"','"&amp;D31&amp;"','"&amp;E31&amp;"','"&amp;F31&amp;"','"&amp;G31&amp;"','"&amp;H31&amp;"');"</f>
-        <v>INSERT INTO MENU VALUES('MENU_0029','1','사용자 권한 부여','MENU_0026','intrAuthInqy3010.do','Y','30','');</v>
+        <v>INSERT INTO MENU VALUES('MENU_0029','1','사용자 권한 부여','MENU_0026','intrRoleInqy3010.do','Y','30','');</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
-        <v>271</v>
+        <v>261</v>
       </c>
       <c r="B32" s="4">
         <v>1</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>212</v>
+        <v>202</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G32" s="4">
         <v>31</v>
@@ -2541,7 +2544,7 @@
   <sheetData>
     <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -2553,13 +2556,13 @@
     </row>
     <row r="2" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="D2" s="6" t="s">
         <v>4</v>
@@ -2579,13 +2582,13 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>260</v>
+        <v>250</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>14</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>262</v>
+        <v>252</v>
       </c>
       <c r="D3" s="4">
         <v>20250520</v>
@@ -2594,7 +2597,7 @@
         <v>80516</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G3" s="4">
         <v>1</v>
@@ -2607,13 +2610,13 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
-        <v>261</v>
+        <v>251</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>263</v>
+        <v>253</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>262</v>
+        <v>252</v>
       </c>
       <c r="D4" s="4">
         <v>20250520</v>
@@ -2622,7 +2625,7 @@
         <v>80525</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G4" s="4">
         <v>2</v>
@@ -2635,13 +2638,13 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>164</v>
+        <v>154</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>196</v>
+        <v>186</v>
       </c>
       <c r="D5" s="4">
         <v>20250520</v>
@@ -2650,7 +2653,7 @@
         <v>80525</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G5" s="4">
         <v>1</v>
@@ -2663,13 +2666,13 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>165</v>
+        <v>155</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>190</v>
+        <v>180</v>
       </c>
       <c r="D6" s="4">
         <v>20250520</v>
@@ -2678,7 +2681,7 @@
         <v>80525</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G6" s="4">
         <v>2</v>
@@ -2691,13 +2694,13 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>190</v>
+        <v>180</v>
       </c>
       <c r="D7" s="4">
         <v>20250520</v>
@@ -2706,7 +2709,7 @@
         <v>80525</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G7" s="4">
         <v>3</v>
@@ -2719,13 +2722,13 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
-        <v>167</v>
+        <v>157</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>153</v>
+        <v>143</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>191</v>
+        <v>181</v>
       </c>
       <c r="D8" s="4">
         <v>20250520</v>
@@ -2734,7 +2737,7 @@
         <v>80525</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G8" s="4">
         <v>1</v>
@@ -2747,13 +2750,13 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
-        <v>168</v>
+        <v>158</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>191</v>
+        <v>181</v>
       </c>
       <c r="D9" s="4">
         <v>20250520</v>
@@ -2762,7 +2765,7 @@
         <v>80525</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G9" s="4">
         <v>2</v>
@@ -2775,13 +2778,13 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>155</v>
+        <v>145</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>191</v>
+        <v>181</v>
       </c>
       <c r="D10" s="4">
         <v>20250520</v>
@@ -2790,7 +2793,7 @@
         <v>80525</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G10" s="4">
         <v>3</v>
@@ -2803,13 +2806,13 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
-        <v>170</v>
+        <v>160</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>156</v>
+        <v>146</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>191</v>
+        <v>181</v>
       </c>
       <c r="D11" s="4">
         <v>20250520</v>
@@ -2818,7 +2821,7 @@
         <v>80525</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G11" s="4">
         <v>4</v>
@@ -2831,13 +2834,13 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
-        <v>171</v>
+        <v>161</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>157</v>
+        <v>147</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>191</v>
+        <v>181</v>
       </c>
       <c r="D12" s="4">
         <v>20250520</v>
@@ -2846,7 +2849,7 @@
         <v>80525</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G12" s="4">
         <v>5</v>
@@ -2859,13 +2862,13 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
-        <v>172</v>
+        <v>162</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>192</v>
+        <v>182</v>
       </c>
       <c r="D13" s="4">
         <v>20250520</v>
@@ -2874,7 +2877,7 @@
         <v>80525</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G13" s="4">
         <v>1</v>
@@ -2887,13 +2890,13 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
-        <v>173</v>
+        <v>163</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>160</v>
+        <v>150</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>192</v>
+        <v>182</v>
       </c>
       <c r="D14" s="4">
         <v>20250520</v>
@@ -2902,7 +2905,7 @@
         <v>80525</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G14" s="4">
         <v>2</v>
@@ -2915,13 +2918,13 @@
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
-        <v>174</v>
+        <v>164</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>161</v>
+        <v>151</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>192</v>
+        <v>182</v>
       </c>
       <c r="D15" s="4">
         <v>20250520</v>
@@ -2930,7 +2933,7 @@
         <v>80525</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G15" s="4">
         <v>3</v>
@@ -2943,13 +2946,13 @@
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>177</v>
+        <v>167</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>193</v>
+        <v>183</v>
       </c>
       <c r="D16" s="4">
         <v>20250520</v>
@@ -2958,7 +2961,7 @@
         <v>80525</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G16" s="4">
         <v>1</v>
@@ -2971,13 +2974,13 @@
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
-        <v>176</v>
+        <v>166</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>162</v>
+        <v>152</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>193</v>
+        <v>183</v>
       </c>
       <c r="D17" s="4">
         <v>20250520</v>
@@ -2986,7 +2989,7 @@
         <v>80525</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G17" s="4">
         <v>2</v>
@@ -2999,13 +3002,13 @@
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
-        <v>178</v>
+        <v>168</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>163</v>
+        <v>153</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>193</v>
+        <v>183</v>
       </c>
       <c r="D18" s="4">
         <v>20250520</v>
@@ -3014,7 +3017,7 @@
         <v>80525</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G18" s="4">
         <v>3</v>
@@ -3027,13 +3030,13 @@
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
-        <v>179</v>
+        <v>169</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>181</v>
+        <v>171</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>194</v>
+        <v>184</v>
       </c>
       <c r="D19" s="4">
         <v>20250520</v>
@@ -3042,7 +3045,7 @@
         <v>80525</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G19" s="4">
         <v>1</v>
@@ -3055,13 +3058,13 @@
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
-        <v>180</v>
+        <v>170</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>182</v>
+        <v>172</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>194</v>
+        <v>184</v>
       </c>
       <c r="D20" s="4">
         <v>20250520</v>
@@ -3070,7 +3073,7 @@
         <v>80525</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G20" s="4">
         <v>2</v>
@@ -3083,13 +3086,13 @@
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>186</v>
+        <v>176</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>195</v>
+        <v>185</v>
       </c>
       <c r="D21" s="4">
         <v>20250520</v>
@@ -3098,7 +3101,7 @@
         <v>80525</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G21" s="4">
         <v>1</v>
@@ -3111,13 +3114,13 @@
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
-        <v>184</v>
+        <v>174</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>187</v>
+        <v>177</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>195</v>
+        <v>185</v>
       </c>
       <c r="D22" s="4">
         <v>20250520</v>
@@ -3126,7 +3129,7 @@
         <v>80525</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G22" s="4">
         <v>2</v>
@@ -3139,13 +3142,13 @@
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="C23" s="4" t="s">
         <v>185</v>
-      </c>
-      <c r="B23" s="4" t="s">
-        <v>188</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>195</v>
       </c>
       <c r="D23" s="4">
         <v>20250520</v>
@@ -3154,7 +3157,7 @@
         <v>80525</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G23" s="4">
         <v>3</v>
@@ -3167,13 +3170,13 @@
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
-        <v>204</v>
+        <v>194</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>205</v>
+        <v>195</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>195</v>
+        <v>185</v>
       </c>
       <c r="D24" s="4">
         <v>20250520</v>
@@ -3182,7 +3185,7 @@
         <v>80525</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G24" s="4">
         <v>4</v>
@@ -3195,13 +3198,13 @@
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
-        <v>198</v>
+        <v>188</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>201</v>
+        <v>191</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>197</v>
+        <v>187</v>
       </c>
       <c r="D25" s="4">
         <v>20250520</v>
@@ -3210,7 +3213,7 @@
         <v>80525</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G25" s="4">
         <v>1</v>
@@ -3223,13 +3226,13 @@
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
-        <v>199</v>
+        <v>189</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>202</v>
+        <v>192</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>197</v>
+        <v>187</v>
       </c>
       <c r="D26" s="4">
         <v>20250520</v>
@@ -3238,7 +3241,7 @@
         <v>80525</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G26" s="4">
         <v>2</v>
@@ -3251,13 +3254,13 @@
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
-        <v>200</v>
+        <v>190</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>203</v>
+        <v>193</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>197</v>
+        <v>187</v>
       </c>
       <c r="D27" s="4">
         <v>20250520</v>
@@ -3266,7 +3269,7 @@
         <v>80525</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G27" s="4">
         <v>3</v>
@@ -3279,13 +3282,13 @@
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
-        <v>264</v>
+        <v>254</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>267</v>
+        <v>257</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>270</v>
+        <v>260</v>
       </c>
       <c r="D28" s="4">
         <v>20250520</v>
@@ -3294,7 +3297,7 @@
         <v>80525</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G28" s="4">
         <v>1</v>
@@ -3307,13 +3310,13 @@
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
-        <v>265</v>
+        <v>255</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>268</v>
+        <v>258</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>270</v>
+        <v>260</v>
       </c>
       <c r="D29" s="4">
         <v>20250520</v>
@@ -3322,7 +3325,7 @@
         <v>80525</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G29" s="4">
         <v>2</v>
@@ -3335,13 +3338,13 @@
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
-        <v>266</v>
+        <v>256</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>269</v>
+        <v>259</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>270</v>
+        <v>260</v>
       </c>
       <c r="D30" s="4">
         <v>20250520</v>
@@ -3350,7 +3353,7 @@
         <v>80525</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G30" s="4">
         <v>3</v>
@@ -3382,7 +3385,7 @@
   <sheetData>
     <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
-        <v>69</v>
+        <v>266</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -3391,10 +3394,10 @@
     </row>
     <row r="2" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
-        <v>32</v>
+        <v>268</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>33</v>
+        <v>271</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>6</v>
@@ -3408,10 +3411,10 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>34</v>
+        <v>270</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>14</v>
@@ -3422,15 +3425,15 @@
       <c r="E3" s="4"/>
       <c r="G3" s="3" t="str">
         <f>"INSERT INTO "&amp;$A$1&amp;" VALUES('"&amp;A3&amp;"','"&amp;B3&amp;"','"&amp;C3&amp;"','"&amp;D3&amp;"','"&amp;E3&amp;"');"</f>
-        <v>INSERT INTO AUTH VALUES('AUTH_0001','관리자 권한','Y','1','');</v>
+        <v>INSERT INTO ROLE VALUES('ROLE_0001','관리자 권한','Y','1','');</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
-        <v>71</v>
+        <v>272</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>14</v>
@@ -3441,7 +3444,7 @@
       <c r="E4" s="4"/>
       <c r="G4" s="3" t="str">
         <f>"INSERT INTO "&amp;$A$1&amp;" VALUES('"&amp;A4&amp;"','"&amp;B4&amp;"','"&amp;C4&amp;"','"&amp;D4&amp;"','"&amp;E4&amp;"');"</f>
-        <v>INSERT INTO AUTH VALUES('AUTH_0002','테스트 권한','Y','2','');</v>
+        <v>INSERT INTO ROLE VALUES('ROLE_0002','테스트 권한','Y','2','');</v>
       </c>
     </row>
   </sheetData>
@@ -3464,7 +3467,7 @@
   <sheetData>
     <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
-        <v>73</v>
+        <v>274</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -3473,7 +3476,7 @@
     </row>
     <row r="2" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
-        <v>32</v>
+        <v>267</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>9</v>
@@ -3490,10 +3493,10 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>34</v>
+        <v>269</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>14</v>
@@ -3504,12 +3507,12 @@
       <c r="E3" s="4"/>
       <c r="G3" s="3" t="str">
         <f>"INSERT INTO "&amp;$A$1&amp;" VALUES('"&amp;A3&amp;"','"&amp;B3&amp;"','"&amp;C3&amp;"','"&amp;D3&amp;"','"&amp;E3&amp;"');"</f>
-        <v>INSERT INTO MENU_AUTH VALUES('AUTH_0001','MENU_0001','Y','1','');</v>
+        <v>INSERT INTO MENU_ROLE VALUES('ROLE_0001','MENU_0001','Y','1','');</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
-        <v>34</v>
+        <v>269</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>16</v>
@@ -3523,12 +3526,12 @@
       <c r="E4" s="4"/>
       <c r="G4" s="3" t="str">
         <f t="shared" ref="G4:G26" si="0">"INSERT INTO "&amp;$A$1&amp;" VALUES('"&amp;A4&amp;"','"&amp;B4&amp;"','"&amp;C4&amp;"','"&amp;D4&amp;"','"&amp;E4&amp;"');"</f>
-        <v>INSERT INTO MENU_AUTH VALUES('AUTH_0001','MENU_0002','Y','2','');</v>
+        <v>INSERT INTO MENU_ROLE VALUES('ROLE_0001','MENU_0002','Y','2','');</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>34</v>
+        <v>269</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>17</v>
@@ -3542,12 +3545,12 @@
       <c r="E5" s="4"/>
       <c r="G5" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>INSERT INTO MENU_AUTH VALUES('AUTH_0001','MENU_0003','Y','3','');</v>
+        <v>INSERT INTO MENU_ROLE VALUES('ROLE_0001','MENU_0003','Y','3','');</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>34</v>
+        <v>269</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>18</v>
@@ -3561,12 +3564,12 @@
       <c r="E6" s="4"/>
       <c r="G6" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>INSERT INTO MENU_AUTH VALUES('AUTH_0001','MENU_0004','Y','4','');</v>
+        <v>INSERT INTO MENU_ROLE VALUES('ROLE_0001','MENU_0004','Y','4','');</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
-        <v>34</v>
+        <v>269</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>15</v>
@@ -3580,12 +3583,12 @@
       <c r="E7" s="4"/>
       <c r="G7" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>INSERT INTO MENU_AUTH VALUES('AUTH_0001','MENU_0005','Y','5','');</v>
+        <v>INSERT INTO MENU_ROLE VALUES('ROLE_0001','MENU_0005','Y','5','');</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
-        <v>34</v>
+        <v>269</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>19</v>
@@ -3599,12 +3602,12 @@
       <c r="E8" s="4"/>
       <c r="G8" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>INSERT INTO MENU_AUTH VALUES('AUTH_0001','MENU_0006','Y','6','');</v>
+        <v>INSERT INTO MENU_ROLE VALUES('ROLE_0001','MENU_0006','Y','6','');</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
-        <v>34</v>
+        <v>269</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>20</v>
@@ -3618,12 +3621,12 @@
       <c r="E9" s="4"/>
       <c r="G9" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>INSERT INTO MENU_AUTH VALUES('AUTH_0001','MENU_0007','Y','7','');</v>
+        <v>INSERT INTO MENU_ROLE VALUES('ROLE_0001','MENU_0007','Y','7','');</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
-        <v>34</v>
+        <v>269</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>21</v>
@@ -3637,12 +3640,12 @@
       <c r="E10" s="4"/>
       <c r="G10" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>INSERT INTO MENU_AUTH VALUES('AUTH_0001','MENU_0008','Y','8','');</v>
+        <v>INSERT INTO MENU_ROLE VALUES('ROLE_0001','MENU_0008','Y','8','');</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
-        <v>34</v>
+        <v>269</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>22</v>
@@ -3656,12 +3659,12 @@
       <c r="E11" s="4"/>
       <c r="G11" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>INSERT INTO MENU_AUTH VALUES('AUTH_0001','MENU_0009','Y','9','');</v>
+        <v>INSERT INTO MENU_ROLE VALUES('ROLE_0001','MENU_0009','Y','9','');</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
-        <v>34</v>
+        <v>269</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>23</v>
@@ -3675,12 +3678,12 @@
       <c r="E12" s="4"/>
       <c r="G12" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>INSERT INTO MENU_AUTH VALUES('AUTH_0001','MENU_0010','Y','10','');</v>
+        <v>INSERT INTO MENU_ROLE VALUES('ROLE_0001','MENU_0010','Y','10','');</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
-        <v>34</v>
+        <v>269</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>24</v>
@@ -3694,12 +3697,12 @@
       <c r="E13" s="4"/>
       <c r="G13" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>INSERT INTO MENU_AUTH VALUES('AUTH_0001','MENU_0011','Y','11','');</v>
+        <v>INSERT INTO MENU_ROLE VALUES('ROLE_0001','MENU_0011','Y','11','');</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
-        <v>34</v>
+        <v>269</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>25</v>
@@ -3713,12 +3716,12 @@
       <c r="E14" s="4"/>
       <c r="G14" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>INSERT INTO MENU_AUTH VALUES('AUTH_0001','MENU_0012','Y','12','');</v>
+        <v>INSERT INTO MENU_ROLE VALUES('ROLE_0001','MENU_0012','Y','12','');</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
-        <v>34</v>
+        <v>269</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>26</v>
@@ -3732,12 +3735,12 @@
       <c r="E15" s="4"/>
       <c r="G15" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>INSERT INTO MENU_AUTH VALUES('AUTH_0001','MENU_0013','Y','13','');</v>
+        <v>INSERT INTO MENU_ROLE VALUES('ROLE_0001','MENU_0013','Y','13','');</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
-        <v>34</v>
+        <v>269</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>27</v>
@@ -3751,12 +3754,12 @@
       <c r="E16" s="4"/>
       <c r="G16" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>INSERT INTO MENU_AUTH VALUES('AUTH_0001','MENU_0014','Y','14','');</v>
+        <v>INSERT INTO MENU_ROLE VALUES('ROLE_0001','MENU_0014','Y','14','');</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
-        <v>34</v>
+        <v>269</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>28</v>
@@ -3770,12 +3773,12 @@
       <c r="E17" s="4"/>
       <c r="G17" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>INSERT INTO MENU_AUTH VALUES('AUTH_0001','MENU_0015','Y','15','');</v>
+        <v>INSERT INTO MENU_ROLE VALUES('ROLE_0001','MENU_0015','Y','15','');</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
-        <v>34</v>
+        <v>269</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>29</v>
@@ -3789,12 +3792,12 @@
       <c r="E18" s="4"/>
       <c r="G18" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>INSERT INTO MENU_AUTH VALUES('AUTH_0001','MENU_0016','Y','16','');</v>
+        <v>INSERT INTO MENU_ROLE VALUES('ROLE_0001','MENU_0016','Y','16','');</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
-        <v>34</v>
+        <v>269</v>
       </c>
       <c r="B19" s="4" t="s">
         <v>30</v>
@@ -3808,15 +3811,15 @@
       <c r="E19" s="4"/>
       <c r="G19" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>INSERT INTO MENU_AUTH VALUES('AUTH_0001','MENU_0017','Y','17','');</v>
+        <v>INSERT INTO MENU_ROLE VALUES('ROLE_0001','MENU_0017','Y','17','');</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
-        <v>34</v>
+        <v>269</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>14</v>
@@ -3827,15 +3830,15 @@
       <c r="E20" s="4"/>
       <c r="G20" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>INSERT INTO MENU_AUTH VALUES('AUTH_0001','MENU_0018','Y','18','');</v>
+        <v>INSERT INTO MENU_ROLE VALUES('ROLE_0001','MENU_0018','Y','18','');</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="B21" s="4" t="s">
         <v>34</v>
-      </c>
-      <c r="B21" s="4" t="s">
-        <v>37</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>14</v>
@@ -3846,15 +3849,15 @@
       <c r="E21" s="4"/>
       <c r="G21" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>INSERT INTO MENU_AUTH VALUES('AUTH_0001','MENU_0019','Y','19','');</v>
+        <v>INSERT INTO MENU_ROLE VALUES('ROLE_0001','MENU_0019','Y','19','');</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
-        <v>34</v>
+        <v>269</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C22" s="4" t="s">
         <v>14</v>
@@ -3865,15 +3868,15 @@
       <c r="E22" s="4"/>
       <c r="G22" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>INSERT INTO MENU_AUTH VALUES('AUTH_0001','MENU_0020','Y','20','');</v>
+        <v>INSERT INTO MENU_ROLE VALUES('ROLE_0001','MENU_0020','Y','20','');</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
-        <v>34</v>
+        <v>269</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C23" s="4" t="s">
         <v>14</v>
@@ -3884,15 +3887,15 @@
       <c r="E23" s="4"/>
       <c r="G23" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>INSERT INTO MENU_AUTH VALUES('AUTH_0001','MENU_0021','Y','21','');</v>
+        <v>INSERT INTO MENU_ROLE VALUES('ROLE_0001','MENU_0021','Y','21','');</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
-        <v>34</v>
+        <v>269</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="C24" s="4" t="s">
         <v>14</v>
@@ -3903,15 +3906,15 @@
       <c r="E24" s="4"/>
       <c r="G24" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>INSERT INTO MENU_AUTH VALUES('AUTH_0001','MENU_0022','Y','22','');</v>
+        <v>INSERT INTO MENU_ROLE VALUES('ROLE_0001','MENU_0022','Y','22','');</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
-        <v>34</v>
+        <v>269</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>14</v>
@@ -3922,15 +3925,15 @@
       <c r="E25" s="4"/>
       <c r="G25" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>INSERT INTO MENU_AUTH VALUES('AUTH_0001','MENU_0023','Y','23','');</v>
+        <v>INSERT INTO MENU_ROLE VALUES('ROLE_0001','MENU_0023','Y','23','');</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
-        <v>34</v>
+        <v>269</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>151</v>
+        <v>141</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>14</v>
@@ -3941,15 +3944,15 @@
       <c r="E26" s="4"/>
       <c r="G26" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>INSERT INTO MENU_AUTH VALUES('AUTH_0001','MENU_0024','Y','24','');</v>
+        <v>INSERT INTO MENU_ROLE VALUES('ROLE_0001','MENU_0024','Y','24','');</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
-        <v>34</v>
+        <v>269</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="C27" s="4" t="s">
         <v>14</v>
@@ -3960,15 +3963,15 @@
       <c r="E27" s="4"/>
       <c r="G27" s="3" t="str">
         <f t="shared" ref="G27" si="1">"INSERT INTO "&amp;$A$1&amp;" VALUES('"&amp;A27&amp;"','"&amp;B27&amp;"','"&amp;C27&amp;"','"&amp;D27&amp;"','"&amp;E27&amp;"');"</f>
-        <v>INSERT INTO MENU_AUTH VALUES('AUTH_0001','MENU_0025','Y','25','');</v>
+        <v>INSERT INTO MENU_ROLE VALUES('ROLE_0001','MENU_0025','Y','25','');</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
-        <v>34</v>
+        <v>269</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>212</v>
+        <v>202</v>
       </c>
       <c r="C28" s="4" t="s">
         <v>14</v>
@@ -3979,15 +3982,15 @@
       <c r="E28" s="4"/>
       <c r="G28" s="3" t="str">
         <f t="shared" ref="G28:G29" si="2">"INSERT INTO "&amp;$A$1&amp;" VALUES('"&amp;A28&amp;"','"&amp;B28&amp;"','"&amp;C28&amp;"','"&amp;D28&amp;"','"&amp;E28&amp;"');"</f>
-        <v>INSERT INTO MENU_AUTH VALUES('AUTH_0001','MENU_0026','Y','26','');</v>
+        <v>INSERT INTO MENU_ROLE VALUES('ROLE_0001','MENU_0026','Y','26','');</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
-        <v>34</v>
+        <v>269</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>213</v>
+        <v>203</v>
       </c>
       <c r="C29" s="4" t="s">
         <v>14</v>
@@ -3998,15 +4001,15 @@
       <c r="E29" s="4"/>
       <c r="G29" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>INSERT INTO MENU_AUTH VALUES('AUTH_0001','MENU_0027','Y','27','');</v>
+        <v>INSERT INTO MENU_ROLE VALUES('ROLE_0001','MENU_0027','Y','27','');</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
-        <v>34</v>
+        <v>269</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>220</v>
+        <v>210</v>
       </c>
       <c r="C30" s="4" t="s">
         <v>14</v>
@@ -4017,15 +4020,15 @@
       <c r="E30" s="4"/>
       <c r="G30" s="3" t="str">
         <f t="shared" ref="G30:G31" si="3">"INSERT INTO "&amp;$A$1&amp;" VALUES('"&amp;A30&amp;"','"&amp;B30&amp;"','"&amp;C30&amp;"','"&amp;D30&amp;"','"&amp;E30&amp;"');"</f>
-        <v>INSERT INTO MENU_AUTH VALUES('AUTH_0001','MENU_0028','Y','28','');</v>
+        <v>INSERT INTO MENU_ROLE VALUES('ROLE_0001','MENU_0028','Y','28','');</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
-        <v>34</v>
+        <v>269</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>221</v>
+        <v>211</v>
       </c>
       <c r="C31" s="4" t="s">
         <v>14</v>
@@ -4036,15 +4039,15 @@
       <c r="E31" s="4"/>
       <c r="G31" s="3" t="str">
         <f t="shared" si="3"/>
-        <v>INSERT INTO MENU_AUTH VALUES('AUTH_0001','MENU_0029','Y','29','');</v>
+        <v>INSERT INTO MENU_ROLE VALUES('ROLE_0001','MENU_0029','Y','29','');</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
-        <v>34</v>
+        <v>269</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>271</v>
+        <v>261</v>
       </c>
       <c r="C32" s="4" t="s">
         <v>14</v>
@@ -4055,7 +4058,7 @@
       <c r="E32" s="4"/>
       <c r="G32" s="3" t="str">
         <f t="shared" ref="G32" si="4">"INSERT INTO "&amp;$A$1&amp;" VALUES('"&amp;A32&amp;"','"&amp;B32&amp;"','"&amp;C32&amp;"','"&amp;D32&amp;"','"&amp;E32&amp;"');"</f>
-        <v>INSERT INTO MENU_AUTH VALUES('AUTH_0001','MENU_0030','Y','30','');</v>
+        <v>INSERT INTO MENU_ROLE VALUES('ROLE_0001','MENU_0030','Y','30','');</v>
       </c>
     </row>
   </sheetData>
@@ -4078,7 +4081,7 @@
   <sheetData>
     <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
-        <v>74</v>
+        <v>273</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -4087,7 +4090,7 @@
     </row>
     <row r="2" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
-        <v>32</v>
+        <v>267</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>0</v>
@@ -4104,13 +4107,13 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>34</v>
+        <v>269</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>206</v>
+        <v>196</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="D3" s="4">
         <v>1</v>
@@ -4118,7 +4121,7 @@
       <c r="E3" s="4"/>
       <c r="G3" s="3" t="str">
         <f>"INSERT INTO "&amp;$A$1&amp;" VALUES('"&amp;A3&amp;"','"&amp;B3&amp;"','"&amp;C3&amp;"','"&amp;D3&amp;"','"&amp;E3&amp;"');"</f>
-        <v>INSERT INTO EMP_AUTH VALUES('AUTH_0001','EMP_0001','Y','1','');</v>
+        <v>INSERT INTO EMP_ROLE VALUES('ROLE_0001','EMP_0001','Y','1','');</v>
       </c>
     </row>
   </sheetData>
@@ -4143,7 +4146,7 @@
   <sheetData>
     <row r="1" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -4163,28 +4166,28 @@
         <v>0</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="D2" s="6" t="s">
         <v>1</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="J2" s="6" t="s">
         <v>2</v>
@@ -4193,41 +4196,41 @@
         <v>3</v>
       </c>
       <c r="L2" s="6" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="M2" s="6" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>
       <c r="I3" s="4" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="K3" s="4" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="L3" s="4">
         <v>20230814</v>
@@ -4261,7 +4264,7 @@
   <sheetData>
     <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -4273,13 +4276,13 @@
     </row>
     <row r="2" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="D2" s="6" t="s">
         <v>4</v>
@@ -4299,20 +4302,20 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>127</v>
+        <v>117</v>
       </c>
       <c r="C3" s="4"/>
       <c r="D3" s="4">
         <v>20230814</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G3" s="4">
         <v>1</v>
@@ -4325,20 +4328,20 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>126</v>
+        <v>116</v>
       </c>
       <c r="C4" s="4"/>
       <c r="D4" s="4">
         <v>20230814</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G4" s="4">
         <v>2</v>
@@ -4351,20 +4354,20 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="C5" s="4"/>
       <c r="D5" s="4">
         <v>20230814</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G5" s="4">
         <v>3</v>
@@ -4377,20 +4380,20 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="C6" s="4"/>
       <c r="D6" s="4">
         <v>20230814</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G6" s="4">
         <v>4</v>
@@ -4403,20 +4406,20 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="C7" s="4"/>
       <c r="D7" s="4">
         <v>20230814</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G7" s="4">
         <v>5</v>
@@ -4429,20 +4432,20 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>131</v>
+        <v>121</v>
       </c>
       <c r="C8" s="4"/>
       <c r="D8" s="4">
         <v>20230814</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G8" s="4">
         <v>6</v>
@@ -4455,20 +4458,20 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
-        <v>121</v>
+        <v>111</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
       <c r="C9" s="4"/>
       <c r="D9" s="4">
         <v>20230814</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G9" s="4">
         <v>7</v>
@@ -4481,20 +4484,20 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
-        <v>122</v>
+        <v>112</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>133</v>
+        <v>123</v>
       </c>
       <c r="C10" s="4"/>
       <c r="D10" s="4">
         <v>20230814</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G10" s="4">
         <v>8</v>
@@ -4507,20 +4510,20 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
-        <v>123</v>
+        <v>113</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="C11" s="4"/>
       <c r="D11" s="4">
         <v>20230814</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G11" s="4">
         <v>9</v>
@@ -4533,20 +4536,20 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
-        <v>124</v>
+        <v>114</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>135</v>
+        <v>125</v>
       </c>
       <c r="C12" s="4"/>
       <c r="D12" s="4">
         <v>20230814</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G12" s="4">
         <v>10</v>
@@ -4559,20 +4562,20 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
-        <v>125</v>
+        <v>115</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
       <c r="C13" s="4"/>
       <c r="D13" s="4">
         <v>20230814</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G13" s="4">
         <v>11</v>
@@ -4585,20 +4588,20 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>137</v>
+        <v>127</v>
       </c>
       <c r="C14" s="4"/>
       <c r="D14" s="4">
         <v>20230814</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G14" s="4">
         <v>12</v>
@@ -4611,20 +4614,20 @@
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>138</v>
+        <v>128</v>
       </c>
       <c r="C15" s="4"/>
       <c r="D15" s="4">
         <v>20230814</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G15" s="4">
         <v>13</v>
@@ -4658,7 +4661,7 @@
   <sheetData>
     <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -4669,10 +4672,10 @@
     </row>
     <row r="2" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>102</v>
+        <v>92</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>4</v>
@@ -4692,19 +4695,19 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="C3" s="4">
         <v>20230814</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F3" s="4">
         <v>1</v>
@@ -4717,19 +4720,19 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="C4" s="4">
         <v>20230814</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F4" s="4">
         <v>2</v>
@@ -4742,19 +4745,19 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="C5" s="4">
         <v>20230814</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F5" s="4">
         <v>3</v>
@@ -4767,19 +4770,19 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="C6" s="4">
         <v>20230814</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F6" s="4">
         <v>4</v>
@@ -4792,19 +4795,19 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="C7" s="4">
         <v>20230814</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F7" s="4">
         <v>5</v>
@@ -4817,19 +4820,19 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="C8" s="4">
         <v>20230814</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F8" s="4">
         <v>6</v>
@@ -4842,19 +4845,19 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="C9" s="4">
         <v>20230814</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F9" s="4">
         <v>7</v>
@@ -4867,19 +4870,19 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="C10" s="4">
         <v>20230814</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F10" s="4">
         <v>8</v>
@@ -4892,19 +4895,19 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="C11" s="4">
         <v>20230814</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F11" s="4">
         <v>9</v>
@@ -4917,19 +4920,19 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="C12" s="4">
         <v>20230814</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F12" s="4">
         <v>10</v>
@@ -4963,7 +4966,7 @@
   <sheetData>
     <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
-        <v>223</v>
+        <v>213</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -4974,16 +4977,16 @@
     </row>
     <row r="2" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
-        <v>224</v>
+        <v>214</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>225</v>
+        <v>215</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>226</v>
+        <v>216</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>227</v>
+        <v>217</v>
       </c>
       <c r="E2" s="6" t="s">
         <v>6</v>
@@ -4997,19 +5000,19 @@
     </row>
     <row r="3" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>232</v>
+        <v>222</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>231</v>
+        <v>221</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>236</v>
+        <v>226</v>
       </c>
       <c r="D3" s="4">
         <v>20250520</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F3" s="4">
         <v>1</v>
@@ -5072,19 +5075,19 @@
     </row>
     <row r="4" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
-        <v>233</v>
+        <v>223</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>228</v>
+        <v>218</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>237</v>
+        <v>227</v>
       </c>
       <c r="D4" s="4">
         <v>20250520</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F4" s="4">
         <v>2</v>
@@ -5149,19 +5152,19 @@
     </row>
     <row r="5" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>234</v>
+        <v>224</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>230</v>
+        <v>220</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>238</v>
+        <v>228</v>
       </c>
       <c r="D5" s="4">
         <v>20250520</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F5" s="4">
         <v>3</v>
@@ -5226,19 +5229,19 @@
     </row>
     <row r="6" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>235</v>
+        <v>225</v>
       </c>
       <c r="B6" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="C6" s="7" t="s">
         <v>229</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>239</v>
       </c>
       <c r="D6" s="4">
         <v>20250520</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F6" s="4">
         <v>4</v>
@@ -5324,7 +5327,7 @@
   <sheetData>
     <row r="1" spans="1:17" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
-        <v>245</v>
+        <v>235</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -5343,31 +5346,31 @@
     </row>
     <row r="2" spans="1:17" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>247</v>
+        <v>237</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>248</v>
+        <v>238</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>249</v>
+        <v>239</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>250</v>
+        <v>240</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>251</v>
+        <v>241</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>252</v>
+        <v>242</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>253</v>
+        <v>243</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>254</v>
+        <v>244</v>
       </c>
       <c r="J2" s="6" t="s">
         <v>0</v>
@@ -5390,13 +5393,13 @@
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>255</v>
+        <v>245</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>256</v>
+        <v>246</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>256</v>
+        <v>246</v>
       </c>
       <c r="D3" s="4">
         <v>19900101</v>
@@ -5405,26 +5408,26 @@
         <v>19901231</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>257</v>
+        <v>247</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="H3" s="8">
         <v>0</v>
       </c>
       <c r="I3" s="4"/>
       <c r="J3" s="4" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="L3" s="5" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="M3" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="N3" s="4">
         <v>1</v>

</xml_diff>

<commit_message>
[수정] CSS 클래스화 처리 (width, height)
</commit_message>
<xml_diff>
--- a/02.프로젝트/01.인트라넷/01.설계/인트라넷 데이터.xlsx
+++ b/02.프로젝트/01.인트라넷/01.설계/인트라넷 데이터.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="9"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="7"/>
   </bookViews>
   <sheets>
     <sheet name="MENU" sheetId="1" state="visible" r:id="rId2"/>
@@ -608,54 +608,54 @@
   <si>
     <t xml:space="preserve">&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;&lt;strong&gt;&lt;span style="font-size:16.0pt"&gt;휴가 신청서&lt;/span&gt;&lt;/strong&gt;&lt;/span&gt;&lt;/p&gt;
 &lt;table align="center" cellspacing="0" class="MsoTableGrid" style="border-collapse:collapse; border:none; width:603px"&gt;
-	&lt;tbody&gt;
-		&lt;tr&gt;
-			&lt;td style="border-color:#0d0d0d; border-style:solid; border-width:1px; height:57px; width:200px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;소&amp;nbsp; 속&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-			&lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:1px solid #0d0d0d; height:57px; width:518px"&gt;
-			&lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
-			&lt;/td&gt;
-		&lt;/tr&gt;
-		&lt;tr&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;성&amp;nbsp; 명&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
-			&lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
-			&lt;/td&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:200px"&gt;직&amp;nbsp; 급&lt;/td&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:518px"&gt;&amp;nbsp;&lt;/td&gt;
-		&lt;/tr&gt;
-		&lt;tr&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;구 &amp;nbsp;분&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-			&lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;( ) 연차 ( ) 병가 ( ) 경조휴가 ( ) 반차 ( ) 기타&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-		&lt;/tr&gt;
-		&lt;tr&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;기 &amp;nbsp;간&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-			&lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;OOOO년 OO월 OO일 ~ OOOO년 OO월 OO일 (O일간)&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-		&lt;/tr&gt;
-		&lt;tr&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;&amp;nbsp; &amp;nbsp; &amp;nbsp; 사&amp;nbsp; 유&lt;/td&gt;
-			&lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;&amp;nbsp;&lt;/td&gt;
-		&lt;/tr&gt;
-		&lt;tr&gt;
-			&lt;td colspan="4" style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:317px; width:603px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;위와 같이 휴가를 신청하오니 허락하여 주시기 바랍니다.&lt;/span&gt;&lt;/p&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;OOOO년 &amp;nbsp;&amp;nbsp;&amp;nbsp;OO월 &amp;nbsp;&amp;nbsp;&amp;nbsp;OO일&lt;/span&gt;&lt;/p&gt;
-			&lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
-			&lt;p style="margin-left:253px; text-align:center"&gt;&lt;span style="font-size:10pt"&gt;성명 : O&amp;nbsp; O&amp;nbsp; O&amp;nbsp; (인)&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-		&lt;/tr&gt;
-	&lt;/tbody&gt;
+ &lt;tbody&gt;
+  &lt;tr&gt;
+   &lt;td style="border-color:#0d0d0d; border-style:solid; border-width:1px; height:57px; width:200px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;소&amp;nbsp; 속&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+   &lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:1px solid #0d0d0d; height:57px; width:518px"&gt;
+   &lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
+   &lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;성&amp;nbsp; 명&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
+   &lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
+   &lt;/td&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:200px"&gt;직&amp;nbsp; 급&lt;/td&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:518px"&gt;&amp;nbsp;&lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;구 &amp;nbsp;분&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+   &lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;( ) 연차 ( ) 병가 ( ) 경조휴가 ( ) 반차 ( ) 기타&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;기 &amp;nbsp;간&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+   &lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;OOOO년 OO월 OO일 ~ OOOO년 OO월 OO일 (O일간)&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td style="border-color:currentcolor #0d0d0d #0d0d0d; border-style:none solid solid; border-width:medium 1px 1px; height:57px; text-align:center; width:200px"&gt;사&amp;nbsp; 유&lt;/td&gt;
+   &lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;&amp;nbsp;&lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td colspan="4" style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:317px; width:603px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;위와 같이 휴가를 신청하오니 허락하여 주시기 바랍니다.&lt;/span&gt;&lt;/p&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;OOOO년 &amp;nbsp;&amp;nbsp;&amp;nbsp;OO월 &amp;nbsp;&amp;nbsp;&amp;nbsp;OO일&lt;/span&gt;&lt;/p&gt;
+   &lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
+   &lt;p style="margin-left:253px; text-align:center"&gt;&lt;span style="font-size:10pt"&gt;성명 : O&amp;nbsp; O&amp;nbsp; O&amp;nbsp; (인)&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+  &lt;/tr&gt;
+ &lt;/tbody&gt;
 &lt;/table&gt;</t>
   </si>
   <si>
@@ -676,56 +676,56 @@
   <si>
     <t xml:space="preserve">&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;&lt;strong&gt;&lt;span style="font-size:16.0pt"&gt;가지급결의서&lt;/span&gt;&lt;/strong&gt;&lt;/span&gt;&lt;/p&gt;
 &lt;table align="center" cellspacing="0" class="MsoTableGrid" style="border-collapse:collapse; border:none; width:603px"&gt;
-	&lt;tbody&gt;
-		&lt;tr&gt;
-			&lt;td style="border-color:#0d0d0d; border-style:solid; border-width:1px; height:57px; width:200px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;소&amp;nbsp; 속&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-			&lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:1px solid #0d0d0d; height:57px; width:518px"&gt;
-			&lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
-			&lt;/td&gt;
-		&lt;/tr&gt;
-		&lt;tr&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:13.3333px"&gt;성&amp;nbsp; 명&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
-			&lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
-			&lt;/td&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:200px"&gt;직&amp;nbsp; 급&lt;/td&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:518px"&gt;&amp;nbsp;&lt;/td&gt;
-		&lt;/tr&gt;
-		&lt;tr&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:13.3333px"&gt;청구 금액&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
-			&lt;p&gt;&lt;span style="font-size:13.3333px"&gt;&amp;nbsp; &amp;nbsp; &amp;nbsp;일금 (\&amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp;)&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:200px"&gt;지급 방법&lt;/td&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:518px"&gt;( ) 현금 ( ) 개인카드 ( ) 전도금&lt;/td&gt;
-		&lt;/tr&gt;
-		&lt;tr&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:13.3333px"&gt;지급 일자&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-			&lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;OOOO년 OO월 OO일&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-		&lt;/tr&gt;
-		&lt;tr&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;&amp;nbsp; &amp;nbsp; &amp;nbsp;사&amp;nbsp; 유&lt;/td&gt;
-			&lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:518px"&gt;&amp;nbsp;&lt;/td&gt;
-		&lt;/tr&gt;
-		&lt;tr&gt;
-			&lt;td colspan="4" style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:317px; width:603px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;위의 금액을 정히 청구하오니 지급하여 주십시오.&lt;/span&gt;&lt;/p&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;OOOO년 &amp;nbsp;&amp;nbsp;&amp;nbsp;OO월 &amp;nbsp;&amp;nbsp;&amp;nbsp;OO일&lt;/span&gt;&lt;/p&gt;
-			&lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
-			&lt;p style="margin-left:253px; text-align:center"&gt;&lt;span style="font-size:10pt"&gt;성명 : O&amp;nbsp; O&amp;nbsp; O&amp;nbsp; (인)&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-		&lt;/tr&gt;
-	&lt;/tbody&gt;
+ &lt;tbody&gt;
+  &lt;tr&gt;
+   &lt;td style="border-color:#0d0d0d; border-style:solid; border-width:1px; height:57px; width:200px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;소&amp;nbsp; 속&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+   &lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:1px solid #0d0d0d; height:57px; width:518px"&gt;
+   &lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
+   &lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:13.3333px"&gt;성&amp;nbsp; 명&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
+   &lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
+   &lt;/td&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:200px"&gt;직&amp;nbsp; 급&lt;/td&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:518px"&gt;&amp;nbsp;&lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:13.3333px"&gt;청구 금액&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
+   &lt;p&gt;&lt;span style="font-size:13.3333px"&gt;&amp;nbsp; &amp;nbsp; &amp;nbsp;일금 (\&amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp;)&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:200px"&gt;지급 방법&lt;/td&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:518px"&gt;( ) 현금 ( ) 개인카드 ( ) 전도금&lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:13.3333px"&gt;지급 일자&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+   &lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;OOOO년 OO월 OO일&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td style="border-color:currentcolor #0d0d0d #0d0d0d; border-style:none solid solid; border-width:medium 1px 1px; height:57px; text-align:center; width:200px"&gt;사&amp;nbsp; 유&lt;/td&gt;
+   &lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:518px"&gt;&amp;nbsp;&lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td colspan="4" style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:317px; width:603px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;위의 금액을 정히 청구하오니 지급하여 주십시오.&lt;/span&gt;&lt;/p&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;OOOO년 &amp;nbsp;&amp;nbsp;&amp;nbsp;OO월 &amp;nbsp;&amp;nbsp;&amp;nbsp;OO일&lt;/span&gt;&lt;/p&gt;
+   &lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
+   &lt;p style="margin-left:253px; text-align:center"&gt;&lt;span style="font-size:10pt"&gt;성명 : O&amp;nbsp; O&amp;nbsp; O&amp;nbsp; (인)&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+  &lt;/tr&gt;
+ &lt;/tbody&gt;
 &lt;/table&gt;</t>
   </si>
   <si>
@@ -744,58 +744,58 @@
     <t>Item</t>
   </si>
   <si>
-    <t xml:space="preserve">&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;&lt;strong&gt;&lt;span style="font-size:16.0pt"&gt;물품반출입 신청서&lt;/span&gt;&lt;/strong&gt;&lt;/span&gt;&lt;/p&gt;
+    <t xml:space="preserve">&lt;p style="text-align:center"&gt;&lt;span style="font-size:21.3333px"&gt;&lt;strong&gt;&amp;nbsp;물품반출입 신청서&lt;/strong&gt;&lt;/span&gt;&lt;/p&gt;
 &lt;table align="center" cellspacing="0" class="MsoTableGrid" style="border-collapse:collapse; border:none; width:603px"&gt;
-	&lt;tbody&gt;
-		&lt;tr&gt;
-			&lt;td style="border-color:#0d0d0d; border-style:solid; border-width:1px; height:57px; width:200px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;소&amp;nbsp; 속&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-			&lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:1px solid #0d0d0d; height:57px; width:518px"&gt;
-			&lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
-			&lt;/td&gt;
-		&lt;/tr&gt;
-		&lt;tr&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:13.3333px"&gt;성&amp;nbsp; 명&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
-			&lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
-			&lt;/td&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:200px"&gt;직&amp;nbsp; 급&lt;/td&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:518px"&gt;&amp;nbsp;&lt;/td&gt;
-		&lt;/tr&gt;
-		&lt;tr&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
-			&lt;p style="text-align:center"&gt;구&amp;nbsp; 분&lt;/p&gt;
-			&lt;/td&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
-			&lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
-			&lt;/td&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:200px"&gt;물&amp;nbsp; 품&lt;/td&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;&amp;nbsp;&lt;/td&gt;
-		&lt;/tr&gt;
-		&lt;tr&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:13.3333px"&gt;반출일&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-			&lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;OOOO년 OO월 OO일&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-		&lt;/tr&gt;
-		&lt;tr&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;&amp;nbsp; &amp;nbsp; &amp;nbsp;사&amp;nbsp; 유&lt;/td&gt;
-			&lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:518px"&gt;&amp;nbsp;&lt;/td&gt;
-		&lt;/tr&gt;
-		&lt;tr&gt;
-			&lt;td colspan="4" style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:317px; width:603px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;위와 같이 물품반출입을 신청하오니 허락하여 주시기 바랍니다.&lt;/span&gt;&lt;/p&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;OOOO년 &amp;nbsp;&amp;nbsp;&amp;nbsp;OO월 &amp;nbsp;&amp;nbsp;&amp;nbsp;OO일&lt;/span&gt;&lt;/p&gt;
-			&lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
-			&lt;p style="margin-left:253px; text-align:center"&gt;&lt;span style="font-size:10pt"&gt;성명 : O&amp;nbsp; O&amp;nbsp; O&amp;nbsp; (인)&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-		&lt;/tr&gt;
-	&lt;/tbody&gt;
+ &lt;tbody&gt;
+  &lt;tr&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:1px solid #0d0d0d; height:57px; width:200px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;소&amp;nbsp; 속&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+   &lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:1px solid #0d0d0d; height:57px; width:518px"&gt;
+   &lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
+   &lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:13.3333px"&gt;성&amp;nbsp; 명&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
+   &lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
+   &lt;/td&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:200px"&gt;직&amp;nbsp; 급&lt;/td&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:518px"&gt;&amp;nbsp;&lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:13.3333px"&gt;구 분&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
+   &lt;p&gt;&lt;span style="font-size:13.3333px"&gt;&amp;nbsp; &amp;nbsp; &amp;nbsp;&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:200px"&gt;물 품&lt;/td&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:518px"&gt;&amp;nbsp;&lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:13.3333px"&gt;반출일&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+   &lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;OOOO년 OO월 OO일&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td style="border-color:currentcolor #0d0d0d #0d0d0d; border-style:none solid solid; border-width:medium 1px 1px; height:57px; text-align:center; width:200px"&gt;사&amp;nbsp; 유&lt;/td&gt;
+   &lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:518px"&gt;&amp;nbsp;&lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td colspan="4" style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:317px; width:603px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;위와 같이 물품반출입을 신청하오니 허락하여 주시기 바랍니다.&lt;/span&gt;&lt;/p&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;OOOO년 &amp;nbsp;&amp;nbsp;&amp;nbsp;OO월 &amp;nbsp;&amp;nbsp;&amp;nbsp;OO일&lt;/span&gt;&lt;/p&gt;
+   &lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
+   &lt;p style="margin-left:253px; text-align:center"&gt;&lt;span style="font-size:10pt"&gt;성명 : O&amp;nbsp; O&amp;nbsp; O&amp;nbsp; (인)&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+  &lt;/tr&gt;
+ &lt;/tbody&gt;
 &lt;/table&gt;</t>
   </si>
   <si>
@@ -814,56 +814,58 @@
     <t>Corp</t>
   </si>
   <si>
-    <t xml:space="preserve">&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;&lt;strong&gt;&lt;span style="font-size:16.0pt"&gt;법인카드 정산서&lt;/span&gt;&lt;/strong&gt;&lt;/span&gt;&lt;/p&gt;
-&lt;table align="center" cellspacing="0" class="MsoTableGrid" style="border-collapse:collapse; border:none; width:603px"&gt;
-	&lt;tbody&gt;
-		&lt;tr&gt;
-			&lt;td style="border-color:#0d0d0d; border-style:solid; border-width:1px; height:57px; width:200px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;소&amp;nbsp; 속&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-			&lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:1px solid #0d0d0d; height:57px; width:518px"&gt;
-			&lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
-			&lt;/td&gt;
-		&lt;/tr&gt;
-		&lt;tr&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:13.3333px"&gt;성&amp;nbsp; 함&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
-			&lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
-			&lt;/td&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:200px"&gt;직&amp;nbsp; 급&lt;/td&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:518px"&gt;&amp;nbsp;&lt;/td&gt;
-		&lt;/tr&gt;
-		&lt;tr&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:13.3333px"&gt;사용 카드&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-			&lt;td colspan="3" rowspan="1" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
-			&lt;p style="text-align:center"&gt;(카드 회사 / 번호)&lt;/p&gt;
-			&lt;/td&gt;
-		&lt;/tr&gt;
-		&lt;tr&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;사용 기간&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-			&lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;OOOO년 OO월 OO일 ~ OOOO년 OO월 OO일&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-		&lt;/tr&gt;
-		&lt;tr&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;&amp;nbsp; 총 사용금액&lt;/td&gt;
-			&lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:518px"&gt;(\&amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; )&lt;/td&gt;
-		&lt;/tr&gt;
-		&lt;tr&gt;
-			&lt;td colspan="4" style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:317px; width:603px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;위와 같이 법인카드 월간 사용금액을 보고하오니 확인하여 주십시오.&lt;/span&gt;&lt;/p&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;OOOO년 &amp;nbsp;&amp;nbsp;&amp;nbsp;OO월 &amp;nbsp;&amp;nbsp;&amp;nbsp;OO일&lt;/span&gt;&lt;/p&gt;
-			&lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
-			&lt;p style="margin-left:253px; text-align:center"&gt;&lt;span style="font-size:10pt"&gt;성명 : O&amp;nbsp; O&amp;nbsp; O&amp;nbsp; (인)&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-		&lt;/tr&gt;
-	&lt;/tbody&gt;
+    <t xml:space="preserve">&lt;p style="text-align:center"&gt;&lt;span style="font-size:21.3333px"&gt;&lt;strong&gt;&amp;nbsp;법인카드 정산서&lt;/strong&gt;&lt;/span&gt;&lt;/p&gt;
+&lt;table align="center" cellspacing="0" class="MsoTableGrid" style="border-collapse:collapse; border-color:currentcolor; border-image:none; border-style:none; border-width:medium; width:503px"&gt;
+ &lt;tbody&gt;
+  &lt;tr&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:1px solid #0d0d0d; height:57px; width:200px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;소&amp;nbsp; 속&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+   &lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:1px solid #0d0d0d; height:57px; width:518px"&gt;
+   &lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
+   &lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:13.3333px"&gt;성&amp;nbsp; 명&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
+   &lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
+   &lt;/td&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:200px"&gt;직&amp;nbsp; 급&lt;/td&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:518px"&gt;&amp;nbsp;&lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:13.3333px"&gt;사용 카드&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+   &lt;td colspan="3" rowspan="1" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
+   &lt;p&gt;&amp;nbsp; &amp;nbsp; &amp;nbsp;(카드 회사 / 카드 번호)&lt;/p&gt;
+   &lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:13.3333px"&gt;사용 일자&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;OOOO년 OO월 OO일&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+   &lt;td style="border-color:currentcolor #0d0d0d #0d0d0d currentcolor; border-style:none solid solid none; border-width:medium 1px 1px medium; height:57px; text-align:center; width:200px"&gt;사용처&lt;/td&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;&amp;nbsp;&lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td style="border-color:currentcolor #0d0d0d #0d0d0d; border-style:none solid solid; border-width:medium 1px 1px; height:57px; text-align:center; width:200px"&gt;&amp;nbsp;사용 목적&lt;/td&gt;
+   &lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:518px"&gt;&amp;nbsp;&lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td colspan="4" style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:317px; width:603px"&gt;
+   &lt;p style="text-align:center"&gt;위와 같이 법인카드 정산 내역을 신청하오니 승인하여 주시기 바랍니다.&lt;/p&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;OOOO년 &amp;nbsp;&amp;nbsp;&amp;nbsp;OO월 &amp;nbsp;&amp;nbsp;&amp;nbsp;OO일&lt;/span&gt;&lt;/p&gt;
+   &lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
+   &lt;p style="margin-left:253px; text-align:center"&gt;&lt;span style="font-size:10pt"&gt;성명 : O&amp;nbsp; O&amp;nbsp; O&amp;nbsp; (인)&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+  &lt;/tr&gt;
+ &lt;/tbody&gt;
 &lt;/table&gt;</t>
   </si>
   <si>
@@ -3274,7 +3276,7 @@
       </c>
       <c r="H24" s="5"/>
       <c r="J24" s="6" t="str">
-        <f t="shared" ref="J24:J30" si="10">"INSERT INTO "&amp;$A$1&amp;" VALUES('"&amp;A24&amp;"','"&amp;B24&amp;"','"&amp;C24&amp;"','"&amp;D24&amp;"','"&amp;E24&amp;"','"&amp;F24&amp;"','"&amp;G24&amp;"','"&amp;H24&amp;"');"</f>
+        <f t="shared" ref="J24:J32" si="10">"INSERT INTO "&amp;$A$1&amp;" VALUES('"&amp;A24&amp;"','"&amp;B24&amp;"','"&amp;C24&amp;"','"&amp;D24&amp;"','"&amp;E24&amp;"','"&amp;F24&amp;"','"&amp;G24&amp;"','"&amp;H24&amp;"');"</f>
         <v xml:space="preserve">INSERT INTO COMMCODE VALUES('STEP_0040','결재취소','Step','20250520','80525','Y','4','');</v>
       </c>
     </row>
@@ -3471,7 +3473,7 @@
       <c r="H31" s="5"/>
       <c r="I31" s="1"/>
       <c r="J31" s="6" t="str">
-        <f>"INSERT INTO "&amp;$A$1&amp;" VALUES('"&amp;A31&amp;"','"&amp;B31&amp;"','"&amp;C31&amp;"','"&amp;D31&amp;"','"&amp;E31&amp;"','"&amp;F31&amp;"','"&amp;G31&amp;"','"&amp;H31&amp;"');"</f>
+        <f t="shared" si="10"/>
         <v xml:space="preserve">INSERT INTO COMMCODE VALUES('PROC_0010','조회','Proc','20250520','80525','Y','1','');</v>
       </c>
     </row>
@@ -3500,7 +3502,7 @@
       <c r="H32" s="5"/>
       <c r="I32" s="1"/>
       <c r="J32" s="6" t="str">
-        <f>"INSERT INTO "&amp;$A$1&amp;" VALUES('"&amp;A32&amp;"','"&amp;B32&amp;"','"&amp;C32&amp;"','"&amp;D32&amp;"','"&amp;E32&amp;"','"&amp;F32&amp;"','"&amp;G32&amp;"','"&amp;H32&amp;"');"</f>
+        <f t="shared" si="10"/>
         <v xml:space="preserve">INSERT INTO COMMCODE VALUES('PROC_0020','처리','Proc','20250520','80525','Y','2','');</v>
       </c>
     </row>
@@ -5208,54 +5210,54 @@
         <f t="shared" ref="K3:K6" si="8">"INSERT INTO "&amp;$A$1&amp;" VALUES('"&amp;A3&amp;"','"&amp;B3&amp;"','"&amp;C3&amp;"','"&amp;D3&amp;"','"&amp;E3&amp;"','"&amp;F3&amp;"','"&amp;G3&amp;"','"&amp;H3&amp;"','"&amp;I3&amp;"');"</f>
         <v xml:space="preserve">INSERT INTO TEMPLATE VALUES('TEMP_0001','휴가 신청서','Leav','&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;&lt;strong&gt;&lt;span style="font-size:16.0pt"&gt;휴가 신청서&lt;/span&gt;&lt;/strong&gt;&lt;/span&gt;&lt;/p&gt;
 &lt;table align="center" cellspacing="0" class="MsoTableGrid" style="border-collapse:collapse; border:none; width:603px"&gt;
-	&lt;tbody&gt;
-		&lt;tr&gt;
-			&lt;td style="border-color:#0d0d0d; border-style:solid; border-width:1px; height:57px; width:200px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;소&amp;nbsp; 속&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-			&lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:1px solid #0d0d0d; height:57px; width:518px"&gt;
-			&lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
-			&lt;/td&gt;
-		&lt;/tr&gt;
-		&lt;tr&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;성&amp;nbsp; 명&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
-			&lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
-			&lt;/td&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:200px"&gt;직&amp;nbsp; 급&lt;/td&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:518px"&gt;&amp;nbsp;&lt;/td&gt;
-		&lt;/tr&gt;
-		&lt;tr&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;구 &amp;nbsp;분&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-			&lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;( ) 연차 ( ) 병가 ( ) 경조휴가 ( ) 반차 ( ) 기타&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-		&lt;/tr&gt;
-		&lt;tr&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;기 &amp;nbsp;간&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-			&lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;OOOO년 OO월 OO일 ~ OOOO년 OO월 OO일 (O일간)&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-		&lt;/tr&gt;
-		&lt;tr&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;&amp;nbsp; &amp;nbsp; &amp;nbsp; 사&amp;nbsp; 유&lt;/td&gt;
-			&lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;&amp;nbsp;&lt;/td&gt;
-		&lt;/tr&gt;
-		&lt;tr&gt;
-			&lt;td colspan="4" style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:317px; width:603px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;위와 같이 휴가를 신청하오니 허락하여 주시기 바랍니다.&lt;/span&gt;&lt;/p&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;OOOO년 &amp;nbsp;&amp;nbsp;&amp;nbsp;OO월 &amp;nbsp;&amp;nbsp;&amp;nbsp;OO일&lt;/span&gt;&lt;/p&gt;
-			&lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
-			&lt;p style="margin-left:253px; text-align:center"&gt;&lt;span style="font-size:10pt"&gt;성명 : O&amp;nbsp; O&amp;nbsp; O&amp;nbsp; (인)&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-		&lt;/tr&gt;
-	&lt;/tbody&gt;
+ &lt;tbody&gt;
+  &lt;tr&gt;
+   &lt;td style="border-color:#0d0d0d; border-style:solid; border-width:1px; height:57px; width:200px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;소&amp;nbsp; 속&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+   &lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:1px solid #0d0d0d; height:57px; width:518px"&gt;
+   &lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
+   &lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;성&amp;nbsp; 명&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
+   &lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
+   &lt;/td&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:200px"&gt;직&amp;nbsp; 급&lt;/td&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:518px"&gt;&amp;nbsp;&lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;구 &amp;nbsp;분&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+   &lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;( ) 연차 ( ) 병가 ( ) 경조휴가 ( ) 반차 ( ) 기타&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;기 &amp;nbsp;간&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+   &lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;OOOO년 OO월 OO일 ~ OOOO년 OO월 OO일 (O일간)&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td style="border-color:currentcolor #0d0d0d #0d0d0d; border-style:none solid solid; border-width:medium 1px 1px; height:57px; text-align:center; width:200px"&gt;사&amp;nbsp; 유&lt;/td&gt;
+   &lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;&amp;nbsp;&lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td colspan="4" style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:317px; width:603px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;위와 같이 휴가를 신청하오니 허락하여 주시기 바랍니다.&lt;/span&gt;&lt;/p&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;OOOO년 &amp;nbsp;&amp;nbsp;&amp;nbsp;OO월 &amp;nbsp;&amp;nbsp;&amp;nbsp;OO일&lt;/span&gt;&lt;/p&gt;
+   &lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
+   &lt;p style="margin-left:253px; text-align:center"&gt;&lt;span style="font-size:10pt"&gt;성명 : O&amp;nbsp; O&amp;nbsp; O&amp;nbsp; (인)&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+  &lt;/tr&gt;
+ &lt;/tbody&gt;
 &lt;/table&gt;','intrAprvInqy1020.do','intrAprvInqy2020.do','Y','1','');</v>
       </c>
     </row>
@@ -5290,56 +5292,56 @@
         <f t="shared" si="8"/>
         <v xml:space="preserve">INSERT INTO TEMPLATE VALUES('TEMP_0002','가지급결의서','Exp','&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;&lt;strong&gt;&lt;span style="font-size:16.0pt"&gt;가지급결의서&lt;/span&gt;&lt;/strong&gt;&lt;/span&gt;&lt;/p&gt;
 &lt;table align="center" cellspacing="0" class="MsoTableGrid" style="border-collapse:collapse; border:none; width:603px"&gt;
-	&lt;tbody&gt;
-		&lt;tr&gt;
-			&lt;td style="border-color:#0d0d0d; border-style:solid; border-width:1px; height:57px; width:200px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;소&amp;nbsp; 속&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-			&lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:1px solid #0d0d0d; height:57px; width:518px"&gt;
-			&lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
-			&lt;/td&gt;
-		&lt;/tr&gt;
-		&lt;tr&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:13.3333px"&gt;성&amp;nbsp; 명&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
-			&lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
-			&lt;/td&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:200px"&gt;직&amp;nbsp; 급&lt;/td&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:518px"&gt;&amp;nbsp;&lt;/td&gt;
-		&lt;/tr&gt;
-		&lt;tr&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:13.3333px"&gt;청구 금액&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
-			&lt;p&gt;&lt;span style="font-size:13.3333px"&gt;&amp;nbsp; &amp;nbsp; &amp;nbsp;일금 (\&amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp;)&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:200px"&gt;지급 방법&lt;/td&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:518px"&gt;( ) 현금 ( ) 개인카드 ( ) 전도금&lt;/td&gt;
-		&lt;/tr&gt;
-		&lt;tr&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:13.3333px"&gt;지급 일자&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-			&lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;OOOO년 OO월 OO일&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-		&lt;/tr&gt;
-		&lt;tr&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;&amp;nbsp; &amp;nbsp; &amp;nbsp;사&amp;nbsp; 유&lt;/td&gt;
-			&lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:518px"&gt;&amp;nbsp;&lt;/td&gt;
-		&lt;/tr&gt;
-		&lt;tr&gt;
-			&lt;td colspan="4" style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:317px; width:603px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;위의 금액을 정히 청구하오니 지급하여 주십시오.&lt;/span&gt;&lt;/p&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;OOOO년 &amp;nbsp;&amp;nbsp;&amp;nbsp;OO월 &amp;nbsp;&amp;nbsp;&amp;nbsp;OO일&lt;/span&gt;&lt;/p&gt;
-			&lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
-			&lt;p style="margin-left:253px; text-align:center"&gt;&lt;span style="font-size:10pt"&gt;성명 : O&amp;nbsp; O&amp;nbsp; O&amp;nbsp; (인)&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-		&lt;/tr&gt;
-	&lt;/tbody&gt;
+ &lt;tbody&gt;
+  &lt;tr&gt;
+   &lt;td style="border-color:#0d0d0d; border-style:solid; border-width:1px; height:57px; width:200px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;소&amp;nbsp; 속&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+   &lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:1px solid #0d0d0d; height:57px; width:518px"&gt;
+   &lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
+   &lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:13.3333px"&gt;성&amp;nbsp; 명&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
+   &lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
+   &lt;/td&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:200px"&gt;직&amp;nbsp; 급&lt;/td&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:518px"&gt;&amp;nbsp;&lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:13.3333px"&gt;청구 금액&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
+   &lt;p&gt;&lt;span style="font-size:13.3333px"&gt;&amp;nbsp; &amp;nbsp; &amp;nbsp;일금 (\&amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp;)&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:200px"&gt;지급 방법&lt;/td&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:518px"&gt;( ) 현금 ( ) 개인카드 ( ) 전도금&lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:13.3333px"&gt;지급 일자&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+   &lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;OOOO년 OO월 OO일&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td style="border-color:currentcolor #0d0d0d #0d0d0d; border-style:none solid solid; border-width:medium 1px 1px; height:57px; text-align:center; width:200px"&gt;사&amp;nbsp; 유&lt;/td&gt;
+   &lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:518px"&gt;&amp;nbsp;&lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td colspan="4" style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:317px; width:603px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;위의 금액을 정히 청구하오니 지급하여 주십시오.&lt;/span&gt;&lt;/p&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;OOOO년 &amp;nbsp;&amp;nbsp;&amp;nbsp;OO월 &amp;nbsp;&amp;nbsp;&amp;nbsp;OO일&lt;/span&gt;&lt;/p&gt;
+   &lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
+   &lt;p style="margin-left:253px; text-align:center"&gt;&lt;span style="font-size:10pt"&gt;성명 : O&amp;nbsp; O&amp;nbsp; O&amp;nbsp; (인)&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+  &lt;/tr&gt;
+ &lt;/tbody&gt;
 &lt;/table&gt;','intrAprvInqy1021.do','intrAprvInqy2021.do','Y','2','');</v>
       </c>
     </row>
@@ -5372,58 +5374,58 @@
       <c r="J5" s="1"/>
       <c r="K5" s="6" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve">INSERT INTO TEMPLATE VALUES('TEMP_0003','물품반출입 신청서','Item','&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;&lt;strong&gt;&lt;span style="font-size:16.0pt"&gt;물품반출입 신청서&lt;/span&gt;&lt;/strong&gt;&lt;/span&gt;&lt;/p&gt;
+        <v xml:space="preserve">INSERT INTO TEMPLATE VALUES('TEMP_0003','물품반출입 신청서','Item','&lt;p style="text-align:center"&gt;&lt;span style="font-size:21.3333px"&gt;&lt;strong&gt;&amp;nbsp;물품반출입 신청서&lt;/strong&gt;&lt;/span&gt;&lt;/p&gt;
 &lt;table align="center" cellspacing="0" class="MsoTableGrid" style="border-collapse:collapse; border:none; width:603px"&gt;
-	&lt;tbody&gt;
-		&lt;tr&gt;
-			&lt;td style="border-color:#0d0d0d; border-style:solid; border-width:1px; height:57px; width:200px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;소&amp;nbsp; 속&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-			&lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:1px solid #0d0d0d; height:57px; width:518px"&gt;
-			&lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
-			&lt;/td&gt;
-		&lt;/tr&gt;
-		&lt;tr&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:13.3333px"&gt;성&amp;nbsp; 명&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
-			&lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
-			&lt;/td&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:200px"&gt;직&amp;nbsp; 급&lt;/td&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:518px"&gt;&amp;nbsp;&lt;/td&gt;
-		&lt;/tr&gt;
-		&lt;tr&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
-			&lt;p style="text-align:center"&gt;구&amp;nbsp; 분&lt;/p&gt;
-			&lt;/td&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
-			&lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
-			&lt;/td&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:200px"&gt;물&amp;nbsp; 품&lt;/td&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;&amp;nbsp;&lt;/td&gt;
-		&lt;/tr&gt;
-		&lt;tr&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:13.3333px"&gt;반출일&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-			&lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;OOOO년 OO월 OO일&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-		&lt;/tr&gt;
-		&lt;tr&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;&amp;nbsp; &amp;nbsp; &amp;nbsp;사&amp;nbsp; 유&lt;/td&gt;
-			&lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:518px"&gt;&amp;nbsp;&lt;/td&gt;
-		&lt;/tr&gt;
-		&lt;tr&gt;
-			&lt;td colspan="4" style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:317px; width:603px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;위와 같이 물품반출입을 신청하오니 허락하여 주시기 바랍니다.&lt;/span&gt;&lt;/p&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;OOOO년 &amp;nbsp;&amp;nbsp;&amp;nbsp;OO월 &amp;nbsp;&amp;nbsp;&amp;nbsp;OO일&lt;/span&gt;&lt;/p&gt;
-			&lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
-			&lt;p style="margin-left:253px; text-align:center"&gt;&lt;span style="font-size:10pt"&gt;성명 : O&amp;nbsp; O&amp;nbsp; O&amp;nbsp; (인)&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-		&lt;/tr&gt;
-	&lt;/tbody&gt;
+ &lt;tbody&gt;
+  &lt;tr&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:1px solid #0d0d0d; height:57px; width:200px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;소&amp;nbsp; 속&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+   &lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:1px solid #0d0d0d; height:57px; width:518px"&gt;
+   &lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
+   &lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:13.3333px"&gt;성&amp;nbsp; 명&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
+   &lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
+   &lt;/td&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:200px"&gt;직&amp;nbsp; 급&lt;/td&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:518px"&gt;&amp;nbsp;&lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:13.3333px"&gt;구 분&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
+   &lt;p&gt;&lt;span style="font-size:13.3333px"&gt;&amp;nbsp; &amp;nbsp; &amp;nbsp;&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:200px"&gt;물 품&lt;/td&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:518px"&gt;&amp;nbsp;&lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:13.3333px"&gt;반출일&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+   &lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;OOOO년 OO월 OO일&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td style="border-color:currentcolor #0d0d0d #0d0d0d; border-style:none solid solid; border-width:medium 1px 1px; height:57px; text-align:center; width:200px"&gt;사&amp;nbsp; 유&lt;/td&gt;
+   &lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:518px"&gt;&amp;nbsp;&lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td colspan="4" style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:317px; width:603px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;위와 같이 물품반출입을 신청하오니 허락하여 주시기 바랍니다.&lt;/span&gt;&lt;/p&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;OOOO년 &amp;nbsp;&amp;nbsp;&amp;nbsp;OO월 &amp;nbsp;&amp;nbsp;&amp;nbsp;OO일&lt;/span&gt;&lt;/p&gt;
+   &lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
+   &lt;p style="margin-left:253px; text-align:center"&gt;&lt;span style="font-size:10pt"&gt;성명 : O&amp;nbsp; O&amp;nbsp; O&amp;nbsp; (인)&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+  &lt;/tr&gt;
+ &lt;/tbody&gt;
 &lt;/table&gt;','intrAprvInqy1022.do','intrAprvInqy2022.do','Y','3','');</v>
       </c>
     </row>
@@ -5456,56 +5458,58 @@
       <c r="J6" s="1"/>
       <c r="K6" s="6" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve">INSERT INTO TEMPLATE VALUES('TEMP_0004','법인카드 정산서','Corp','&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;&lt;strong&gt;&lt;span style="font-size:16.0pt"&gt;법인카드 정산서&lt;/span&gt;&lt;/strong&gt;&lt;/span&gt;&lt;/p&gt;
-&lt;table align="center" cellspacing="0" class="MsoTableGrid" style="border-collapse:collapse; border:none; width:603px"&gt;
-	&lt;tbody&gt;
-		&lt;tr&gt;
-			&lt;td style="border-color:#0d0d0d; border-style:solid; border-width:1px; height:57px; width:200px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;소&amp;nbsp; 속&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-			&lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:1px solid #0d0d0d; height:57px; width:518px"&gt;
-			&lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
-			&lt;/td&gt;
-		&lt;/tr&gt;
-		&lt;tr&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:13.3333px"&gt;성&amp;nbsp; 함&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
-			&lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
-			&lt;/td&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:200px"&gt;직&amp;nbsp; 급&lt;/td&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:518px"&gt;&amp;nbsp;&lt;/td&gt;
-		&lt;/tr&gt;
-		&lt;tr&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:13.3333px"&gt;사용 카드&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-			&lt;td colspan="3" rowspan="1" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
-			&lt;p style="text-align:center"&gt;(카드 회사 / 번호)&lt;/p&gt;
-			&lt;/td&gt;
-		&lt;/tr&gt;
-		&lt;tr&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;사용 기간&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-			&lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;OOOO년 OO월 OO일 ~ OOOO년 OO월 OO일&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-		&lt;/tr&gt;
-		&lt;tr&gt;
-			&lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;&amp;nbsp; 총 사용금액&lt;/td&gt;
-			&lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:518px"&gt;(\&amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; )&lt;/td&gt;
-		&lt;/tr&gt;
-		&lt;tr&gt;
-			&lt;td colspan="4" style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:317px; width:603px"&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;위와 같이 법인카드 월간 사용금액을 보고하오니 확인하여 주십시오.&lt;/span&gt;&lt;/p&gt;
-			&lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;OOOO년 &amp;nbsp;&amp;nbsp;&amp;nbsp;OO월 &amp;nbsp;&amp;nbsp;&amp;nbsp;OO일&lt;/span&gt;&lt;/p&gt;
-			&lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
-			&lt;p style="margin-left:253px; text-align:center"&gt;&lt;span style="font-size:10pt"&gt;성명 : O&amp;nbsp; O&amp;nbsp; O&amp;nbsp; (인)&lt;/span&gt;&lt;/p&gt;
-			&lt;/td&gt;
-		&lt;/tr&gt;
-	&lt;/tbody&gt;
+        <v xml:space="preserve">INSERT INTO TEMPLATE VALUES('TEMP_0004','법인카드 정산서','Corp','&lt;p style="text-align:center"&gt;&lt;span style="font-size:21.3333px"&gt;&lt;strong&gt;&amp;nbsp;법인카드 정산서&lt;/strong&gt;&lt;/span&gt;&lt;/p&gt;
+&lt;table align="center" cellspacing="0" class="MsoTableGrid" style="border-collapse:collapse; border-color:currentcolor; border-image:none; border-style:none; border-width:medium; width:503px"&gt;
+ &lt;tbody&gt;
+  &lt;tr&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:1px solid #0d0d0d; height:57px; width:200px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;소&amp;nbsp; 속&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+   &lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:1px solid #0d0d0d; height:57px; width:518px"&gt;
+   &lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
+   &lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:13.3333px"&gt;성&amp;nbsp; 명&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
+   &lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
+   &lt;/td&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:200px"&gt;직&amp;nbsp; 급&lt;/td&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:518px"&gt;&amp;nbsp;&lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:13.3333px"&gt;사용 카드&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+   &lt;td colspan="3" rowspan="1" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
+   &lt;p&gt;&amp;nbsp; &amp;nbsp; &amp;nbsp;(카드 회사 / 카드 번호)&lt;/p&gt;
+   &lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:200px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:13.3333px"&gt;사용 일자&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;OOOO년 OO월 OO일&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+   &lt;td style="border-color:currentcolor #0d0d0d #0d0d0d currentcolor; border-style:none solid solid none; border-width:medium 1px 1px medium; height:57px; text-align:center; width:200px"&gt;사용처&lt;/td&gt;
+   &lt;td style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; width:518px"&gt;&amp;nbsp;&lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td style="border-color:currentcolor #0d0d0d #0d0d0d; border-style:none solid solid; border-width:medium 1px 1px; height:57px; text-align:center; width:200px"&gt;&amp;nbsp;사용 목적&lt;/td&gt;
+   &lt;td colspan="3" style="border-bottom:1px solid #0d0d0d; border-left:none; border-right:1px solid #0d0d0d; border-top:none; height:57px; text-align:center; width:518px"&gt;&amp;nbsp;&lt;/td&gt;
+  &lt;/tr&gt;
+  &lt;tr&gt;
+   &lt;td colspan="4" style="border-bottom:1px solid #0d0d0d; border-left:1px solid #0d0d0d; border-right:1px solid #0d0d0d; border-top:none; height:317px; width:603px"&gt;
+   &lt;p style="text-align:center"&gt;위와 같이 법인카드 정산 내역을 신청하오니 승인하여 주시기 바랍니다.&lt;/p&gt;
+   &lt;p style="text-align:center"&gt;&lt;span style="font-size:10pt"&gt;OOOO년 &amp;nbsp;&amp;nbsp;&amp;nbsp;OO월 &amp;nbsp;&amp;nbsp;&amp;nbsp;OO일&lt;/span&gt;&lt;/p&gt;
+   &lt;p style="text-align:center"&gt;&amp;nbsp;&lt;/p&gt;
+   &lt;p style="margin-left:253px; text-align:center"&gt;&lt;span style="font-size:10pt"&gt;성명 : O&amp;nbsp; O&amp;nbsp; O&amp;nbsp; (인)&lt;/span&gt;&lt;/p&gt;
+   &lt;/td&gt;
+  &lt;/tr&gt;
+ &lt;/tbody&gt;
 &lt;/table&gt;','intrAprvInqy1023.do','intrAprvInqy2023.do','Y','4','');</v>
       </c>
     </row>

</xml_diff>